<commit_message>
feat: dem nguoc linh hoat, nhom theo tuan, gio su kien, member tu doi trang thai
- Dem nguoc tuan/ngay khi con xa, dong ho giay khi <24h; gom viec theo nhom thoi gian (Qua han / Tuan nay / Tuan sau / 2-3 tuan / 1 thang / Da xong)
- Nhan hien thi: Han day du (Vao HH:MM - Thu X), tien to Ban, X su kien
- Gio cu the cua su kien (eventStartTime): import cot Gio tu Excel, lam deadline nhip Trong, hien dong Su kien tren the viec; trong -> 17:30
- Moi thanh vien tu doi trang thai viec cua minh qua PATCH /api/tasks/<id>/status (mien rao ghi, chi doi truong status); xoa/nhac van admin-only
- Tab Su kien: to xanh + huy hieu Co viec cua ban cho viec minh phu trach
- Cap nhat template them cot Gio; bump cache v=20260605f

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/mau-ke-hoach-su-kien.xlsx
+++ b/mau-ke-hoach-su-kien.xlsx
@@ -27,20 +27,14 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001A4D6D"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -57,7 +51,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -423,13 +417,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -445,10 +440,15 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Giờ</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Sự kiện / Chương trình</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
@@ -465,10 +465,15 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>08:00</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>Khóa Bồi dưỡng Truyền thông Công giáo</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -481,10 +486,15 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Thông báo chuẩn bị Rước Lễ Lần Đầu</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -497,10 +507,15 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>05:30</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>Thánh Lễ Lãnh nhận Bí Tích Rước Lễ Lần Đầu</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -511,14 +526,15 @@
           <t>03.06–03.07.2026</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" t="inlineStr"/>
+      <c r="D5" t="inlineStr">
         <is>
           <t>Chương trình Hè 2026</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Cả tháng</t>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Cả tháng (không cố định giờ)</t>
         </is>
       </c>
     </row>

</xml_diff>